<commit_message>
fix(templates): count concrete rebar sticks from the cut list
The Slab Takeoff sheet ordered ROUNDUP(total rebar LF ÷ stick length),
which undercounts: steel comes in whole sticks, so a 19½ ft bar takes a
whole 20 ft stick and its drop is not another bar. The sample driveway
came to 49 sticks where the cut list needs 51.

Each slab row now has a Rebar sticks column: every piece of a run but the
last is a full stick, and the end pieces are cut as many to a stick as
fit. The order quantity sums that column. The sample goes from 58 to 62
sticks (driveway 51, apron 11), matching the rebar calculator's nesting
per slab; checked in LibreOffice at 20 ft and 40 ft stock.

The sheet widens to 13 columns, so the assumption values move from L to
M. The landing page FAQ and method paragraph had the same divide-by-
stick-length advice and now explain the cut-list count.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015qp8CUng2McijMKRZYtSLd
</commit_message>
<xml_diff>
--- a/public/templates-files/concrete-estimate-template.xlsx
+++ b/public/templates-files/concrete-estimate-template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="174">
   <si>
     <t>Concrete Estimate</t>
   </si>
@@ -238,6 +238,9 @@
     <t>REBAR LF INCL. LAPS</t>
   </si>
   <si>
+    <t>REBAR STICKS</t>
+  </si>
+  <si>
     <t>CONTROL JOINTS (LF)</t>
   </si>
   <si>
@@ -361,7 +364,7 @@
     <t>LF</t>
   </si>
   <si>
-    <t>Rebar sticks at the stock length</t>
+    <t>Rebar sticks at the stock length — from the cut list</t>
   </si>
   <si>
     <t>PC</t>
@@ -391,7 +394,7 @@
     <t>GAL</t>
   </si>
   <si>
-    <t>CY = length × width × (thickness in inches ÷ 12) ÷ 27. Bars each way = ROUNDUP(clear span ÷ spacing) + 1, plus a lap at every splice. Joint spacing in feet of 2–3 × the slab thickness in inches is a common rule of thumb for plain flatwork, not a code value; keep panels close to square.</t>
+    <t>CY = length × width × (thickness in inches ÷ 12) ÷ 27. Bars each way = ROUNDUP(clear span ÷ spacing) + 1, plus a lap at every splice. Sticks count each run’s full sticks plus its end pieces, cut as many to a stick as fit — more than LF ÷ stick length, because a 19½ ft bar takes a whole 20 ft stick. Joint spacing in feet of 2–3 × the slab thickness in inches is a common rule of thumb for plain flatwork, not a code value; keep panels close to square.</t>
   </si>
   <si>
     <t>Pro tip: check the grade before you trust the depth. A slab that runs ½" thick over 1,000 sq ft uses about 1.5 CY more than you priced. Footings, walls, structural slabs and anything load-bearing follow the engineer’s drawings and local code.</t>
@@ -2131,14 +2134,18 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="3" width="8" customWidth="1"/>
-    <col min="4" max="5" width="7.5" customWidth="1"/>
-    <col min="6" max="6" width="8" customWidth="1"/>
-    <col min="10" max="12" width="10" customWidth="1"/>
+    <col min="2" max="3" width="7.5" customWidth="1"/>
+    <col min="4" max="5" width="7" customWidth="1"/>
+    <col min="6" max="6" width="7.5" customWidth="1"/>
+    <col min="7" max="7" width="8" customWidth="1"/>
+    <col min="8" max="9" width="8.5" customWidth="1"/>
+    <col min="10" max="11" width="9.5" customWidth="1"/>
+    <col min="12" max="12" width="8.5" customWidth="1"/>
+    <col min="13" max="13" width="9.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -2151,7 +2158,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" ht="6" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" ht="6" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2164,6 +2171,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
@@ -2171,7 +2179,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>62</v>
       </c>
@@ -2208,10 +2216,13 @@
       <c r="L6" s="14" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B7" s="39">
         <v>44</v>
@@ -2223,7 +2234,7 @@
         <v>5</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F7" s="39">
         <v>10</v>
@@ -2238,18 +2249,21 @@
         <f>IF(G7="","",2*(B7+C7))</f>
       </c>
       <c r="J7" s="43">
-        <f>IF(AND(G7&lt;&gt;"",UPPER(E7)="Y"),(ROUNDUP((C7-2*$L$19/12)*12/$L$18,0)+1)&amp;" / "&amp;(ROUNDUP((B7-2*$L$19/12)*12/$L$18,0)+1),"")</f>
+        <f>IF(AND(G7&lt;&gt;"",UPPER(E7)="Y"),(ROUNDUP((C7-2*$M$19/12)*12/$M$18,0)+1)&amp;" / "&amp;(ROUNDUP((B7-2*$M$19/12)*12/$M$18,0)+1),"")</f>
       </c>
       <c r="K7" s="41">
-        <f>IF(AND(G7&lt;&gt;"",UPPER(E7)="Y"),(ROUNDUP((C7-2*$L$19/12)*12/$L$18,0)+1)*((B7-2*$L$19/12)+(MAX(1,ROUNDUP(((B7-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12)+(ROUNDUP((B7-2*$L$19/12)*12/$L$18,0)+1)*((C7-2*$L$19/12)+(MAX(1,ROUNDUP(((C7-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12),"")</f>
+        <f>IF(AND(G7&lt;&gt;"",UPPER(E7)="Y"),(ROUNDUP((C7-2*$M$19/12)*12/$M$18,0)+1)*((B7-2*$M$19/12)+(MAX(1,ROUNDUP(((B7-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12)+(ROUNDUP((B7-2*$M$19/12)*12/$M$18,0)+1)*((C7-2*$M$19/12)+(MAX(1,ROUNDUP(((C7-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12),"")</f>
       </c>
       <c r="L7" s="41">
+        <f>IF(AND(G7&lt;&gt;"",UPPER(E7)="Y"),(ROUNDUP((C7-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((B7-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((C7-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((B7-2*$M$19/12)-(MAX(1,ROUNDUP(((B7-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0)+(ROUNDUP((B7-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((C7-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((B7-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((C7-2*$M$19/12)-(MAX(1,ROUNDUP(((C7-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0),"")</f>
+      </c>
+      <c r="M7" s="41">
         <f>IF(OR(G7="",N(F7)&lt;=0),"",(ROUNDUP(B7/F7,0)-1)*C7+(ROUNDUP(C7/F7,0)-1)*B7)</f>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B8" s="39">
         <v>20</v>
@@ -2261,7 +2275,7 @@
         <v>6</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F8" s="39">
         <v>10</v>
@@ -2276,18 +2290,21 @@
         <f>IF(G8="","",2*(B8+C8))</f>
       </c>
       <c r="J8" s="43">
-        <f>IF(AND(G8&lt;&gt;"",UPPER(E8)="Y"),(ROUNDUP((C8-2*$L$19/12)*12/$L$18,0)+1)&amp;" / "&amp;(ROUNDUP((B8-2*$L$19/12)*12/$L$18,0)+1),"")</f>
+        <f>IF(AND(G8&lt;&gt;"",UPPER(E8)="Y"),(ROUNDUP((C8-2*$M$19/12)*12/$M$18,0)+1)&amp;" / "&amp;(ROUNDUP((B8-2*$M$19/12)*12/$M$18,0)+1),"")</f>
       </c>
       <c r="K8" s="41">
-        <f>IF(AND(G8&lt;&gt;"",UPPER(E8)="Y"),(ROUNDUP((C8-2*$L$19/12)*12/$L$18,0)+1)*((B8-2*$L$19/12)+(MAX(1,ROUNDUP(((B8-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12)+(ROUNDUP((B8-2*$L$19/12)*12/$L$18,0)+1)*((C8-2*$L$19/12)+(MAX(1,ROUNDUP(((C8-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12),"")</f>
+        <f>IF(AND(G8&lt;&gt;"",UPPER(E8)="Y"),(ROUNDUP((C8-2*$M$19/12)*12/$M$18,0)+1)*((B8-2*$M$19/12)+(MAX(1,ROUNDUP(((B8-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12)+(ROUNDUP((B8-2*$M$19/12)*12/$M$18,0)+1)*((C8-2*$M$19/12)+(MAX(1,ROUNDUP(((C8-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12),"")</f>
       </c>
       <c r="L8" s="41">
+        <f>IF(AND(G8&lt;&gt;"",UPPER(E8)="Y"),(ROUNDUP((C8-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((B8-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((C8-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((B8-2*$M$19/12)-(MAX(1,ROUNDUP(((B8-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0)+(ROUNDUP((B8-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((C8-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((B8-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((C8-2*$M$19/12)-(MAX(1,ROUNDUP(((C8-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0),"")</f>
+      </c>
+      <c r="M8" s="41">
         <f>IF(OR(G8="",N(F8)&lt;=0),"",(ROUNDUP(B8/F8,0)-1)*C8+(ROUNDUP(C8/F8,0)-1)*B8)</f>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B9" s="39">
         <v>28</v>
@@ -2299,7 +2316,7 @@
         <v>4</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F9" s="39">
         <v>4</v>
@@ -2314,16 +2331,19 @@
         <f>IF(G9="","",2*(B9+C9))</f>
       </c>
       <c r="J9" s="43">
-        <f>IF(AND(G9&lt;&gt;"",UPPER(E9)="Y"),(ROUNDUP((C9-2*$L$19/12)*12/$L$18,0)+1)&amp;" / "&amp;(ROUNDUP((B9-2*$L$19/12)*12/$L$18,0)+1),"")</f>
+        <f>IF(AND(G9&lt;&gt;"",UPPER(E9)="Y"),(ROUNDUP((C9-2*$M$19/12)*12/$M$18,0)+1)&amp;" / "&amp;(ROUNDUP((B9-2*$M$19/12)*12/$M$18,0)+1),"")</f>
       </c>
       <c r="K9" s="41">
-        <f>IF(AND(G9&lt;&gt;"",UPPER(E9)="Y"),(ROUNDUP((C9-2*$L$19/12)*12/$L$18,0)+1)*((B9-2*$L$19/12)+(MAX(1,ROUNDUP(((B9-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12)+(ROUNDUP((B9-2*$L$19/12)*12/$L$18,0)+1)*((C9-2*$L$19/12)+(MAX(1,ROUNDUP(((C9-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12),"")</f>
+        <f>IF(AND(G9&lt;&gt;"",UPPER(E9)="Y"),(ROUNDUP((C9-2*$M$19/12)*12/$M$18,0)+1)*((B9-2*$M$19/12)+(MAX(1,ROUNDUP(((B9-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12)+(ROUNDUP((B9-2*$M$19/12)*12/$M$18,0)+1)*((C9-2*$M$19/12)+(MAX(1,ROUNDUP(((C9-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12),"")</f>
       </c>
       <c r="L9" s="41">
+        <f>IF(AND(G9&lt;&gt;"",UPPER(E9)="Y"),(ROUNDUP((C9-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((B9-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((C9-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((B9-2*$M$19/12)-(MAX(1,ROUNDUP(((B9-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0)+(ROUNDUP((B9-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((C9-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((B9-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((C9-2*$M$19/12)-(MAX(1,ROUNDUP(((C9-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0),"")</f>
+      </c>
+      <c r="M9" s="41">
         <f>IF(OR(G9="",N(F9)&lt;=0),"",(ROUNDUP(B9/F9,0)-1)*C9+(ROUNDUP(C9/F9,0)-1)*B9)</f>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="38"/>
       <c r="B10" s="39"/>
       <c r="C10" s="39"/>
@@ -2340,16 +2360,19 @@
         <f>IF(G10="","",2*(B10+C10))</f>
       </c>
       <c r="J10" s="43">
-        <f>IF(AND(G10&lt;&gt;"",UPPER(E10)="Y"),(ROUNDUP((C10-2*$L$19/12)*12/$L$18,0)+1)&amp;" / "&amp;(ROUNDUP((B10-2*$L$19/12)*12/$L$18,0)+1),"")</f>
+        <f>IF(AND(G10&lt;&gt;"",UPPER(E10)="Y"),(ROUNDUP((C10-2*$M$19/12)*12/$M$18,0)+1)&amp;" / "&amp;(ROUNDUP((B10-2*$M$19/12)*12/$M$18,0)+1),"")</f>
       </c>
       <c r="K10" s="41">
-        <f>IF(AND(G10&lt;&gt;"",UPPER(E10)="Y"),(ROUNDUP((C10-2*$L$19/12)*12/$L$18,0)+1)*((B10-2*$L$19/12)+(MAX(1,ROUNDUP(((B10-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12)+(ROUNDUP((B10-2*$L$19/12)*12/$L$18,0)+1)*((C10-2*$L$19/12)+(MAX(1,ROUNDUP(((C10-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12),"")</f>
+        <f>IF(AND(G10&lt;&gt;"",UPPER(E10)="Y"),(ROUNDUP((C10-2*$M$19/12)*12/$M$18,0)+1)*((B10-2*$M$19/12)+(MAX(1,ROUNDUP(((B10-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12)+(ROUNDUP((B10-2*$M$19/12)*12/$M$18,0)+1)*((C10-2*$M$19/12)+(MAX(1,ROUNDUP(((C10-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12),"")</f>
       </c>
       <c r="L10" s="41">
+        <f>IF(AND(G10&lt;&gt;"",UPPER(E10)="Y"),(ROUNDUP((C10-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((B10-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((C10-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((B10-2*$M$19/12)-(MAX(1,ROUNDUP(((B10-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0)+(ROUNDUP((B10-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((C10-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((B10-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((C10-2*$M$19/12)-(MAX(1,ROUNDUP(((C10-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0),"")</f>
+      </c>
+      <c r="M10" s="41">
         <f>IF(OR(G10="",N(F10)&lt;=0),"",(ROUNDUP(B10/F10,0)-1)*C10+(ROUNDUP(C10/F10,0)-1)*B10)</f>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="38"/>
       <c r="B11" s="39"/>
       <c r="C11" s="39"/>
@@ -2366,16 +2389,19 @@
         <f>IF(G11="","",2*(B11+C11))</f>
       </c>
       <c r="J11" s="43">
-        <f>IF(AND(G11&lt;&gt;"",UPPER(E11)="Y"),(ROUNDUP((C11-2*$L$19/12)*12/$L$18,0)+1)&amp;" / "&amp;(ROUNDUP((B11-2*$L$19/12)*12/$L$18,0)+1),"")</f>
+        <f>IF(AND(G11&lt;&gt;"",UPPER(E11)="Y"),(ROUNDUP((C11-2*$M$19/12)*12/$M$18,0)+1)&amp;" / "&amp;(ROUNDUP((B11-2*$M$19/12)*12/$M$18,0)+1),"")</f>
       </c>
       <c r="K11" s="41">
-        <f>IF(AND(G11&lt;&gt;"",UPPER(E11)="Y"),(ROUNDUP((C11-2*$L$19/12)*12/$L$18,0)+1)*((B11-2*$L$19/12)+(MAX(1,ROUNDUP(((B11-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12)+(ROUNDUP((B11-2*$L$19/12)*12/$L$18,0)+1)*((C11-2*$L$19/12)+(MAX(1,ROUNDUP(((C11-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12),"")</f>
+        <f>IF(AND(G11&lt;&gt;"",UPPER(E11)="Y"),(ROUNDUP((C11-2*$M$19/12)*12/$M$18,0)+1)*((B11-2*$M$19/12)+(MAX(1,ROUNDUP(((B11-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12)+(ROUNDUP((B11-2*$M$19/12)*12/$M$18,0)+1)*((C11-2*$M$19/12)+(MAX(1,ROUNDUP(((C11-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12),"")</f>
       </c>
       <c r="L11" s="41">
+        <f>IF(AND(G11&lt;&gt;"",UPPER(E11)="Y"),(ROUNDUP((C11-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((B11-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((C11-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((B11-2*$M$19/12)-(MAX(1,ROUNDUP(((B11-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0)+(ROUNDUP((B11-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((C11-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((B11-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((C11-2*$M$19/12)-(MAX(1,ROUNDUP(((C11-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0),"")</f>
+      </c>
+      <c r="M11" s="41">
         <f>IF(OR(G11="",N(F11)&lt;=0),"",(ROUNDUP(B11/F11,0)-1)*C11+(ROUNDUP(C11/F11,0)-1)*B11)</f>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="38"/>
       <c r="B12" s="39"/>
       <c r="C12" s="39"/>
@@ -2392,16 +2418,19 @@
         <f>IF(G12="","",2*(B12+C12))</f>
       </c>
       <c r="J12" s="43">
-        <f>IF(AND(G12&lt;&gt;"",UPPER(E12)="Y"),(ROUNDUP((C12-2*$L$19/12)*12/$L$18,0)+1)&amp;" / "&amp;(ROUNDUP((B12-2*$L$19/12)*12/$L$18,0)+1),"")</f>
+        <f>IF(AND(G12&lt;&gt;"",UPPER(E12)="Y"),(ROUNDUP((C12-2*$M$19/12)*12/$M$18,0)+1)&amp;" / "&amp;(ROUNDUP((B12-2*$M$19/12)*12/$M$18,0)+1),"")</f>
       </c>
       <c r="K12" s="41">
-        <f>IF(AND(G12&lt;&gt;"",UPPER(E12)="Y"),(ROUNDUP((C12-2*$L$19/12)*12/$L$18,0)+1)*((B12-2*$L$19/12)+(MAX(1,ROUNDUP(((B12-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12)+(ROUNDUP((B12-2*$L$19/12)*12/$L$18,0)+1)*((C12-2*$L$19/12)+(MAX(1,ROUNDUP(((C12-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12),"")</f>
+        <f>IF(AND(G12&lt;&gt;"",UPPER(E12)="Y"),(ROUNDUP((C12-2*$M$19/12)*12/$M$18,0)+1)*((B12-2*$M$19/12)+(MAX(1,ROUNDUP(((B12-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12)+(ROUNDUP((B12-2*$M$19/12)*12/$M$18,0)+1)*((C12-2*$M$19/12)+(MAX(1,ROUNDUP(((C12-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12),"")</f>
       </c>
       <c r="L12" s="41">
+        <f>IF(AND(G12&lt;&gt;"",UPPER(E12)="Y"),(ROUNDUP((C12-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((B12-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((C12-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((B12-2*$M$19/12)-(MAX(1,ROUNDUP(((B12-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0)+(ROUNDUP((B12-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((C12-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((B12-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((C12-2*$M$19/12)-(MAX(1,ROUNDUP(((C12-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0),"")</f>
+      </c>
+      <c r="M12" s="41">
         <f>IF(OR(G12="",N(F12)&lt;=0),"",(ROUNDUP(B12/F12,0)-1)*C12+(ROUNDUP(C12/F12,0)-1)*B12)</f>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="38"/>
       <c r="B13" s="39"/>
       <c r="C13" s="39"/>
@@ -2418,16 +2447,19 @@
         <f>IF(G13="","",2*(B13+C13))</f>
       </c>
       <c r="J13" s="43">
-        <f>IF(AND(G13&lt;&gt;"",UPPER(E13)="Y"),(ROUNDUP((C13-2*$L$19/12)*12/$L$18,0)+1)&amp;" / "&amp;(ROUNDUP((B13-2*$L$19/12)*12/$L$18,0)+1),"")</f>
+        <f>IF(AND(G13&lt;&gt;"",UPPER(E13)="Y"),(ROUNDUP((C13-2*$M$19/12)*12/$M$18,0)+1)&amp;" / "&amp;(ROUNDUP((B13-2*$M$19/12)*12/$M$18,0)+1),"")</f>
       </c>
       <c r="K13" s="41">
-        <f>IF(AND(G13&lt;&gt;"",UPPER(E13)="Y"),(ROUNDUP((C13-2*$L$19/12)*12/$L$18,0)+1)*((B13-2*$L$19/12)+(MAX(1,ROUNDUP(((B13-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12)+(ROUNDUP((B13-2*$L$19/12)*12/$L$18,0)+1)*((C13-2*$L$19/12)+(MAX(1,ROUNDUP(((C13-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12),"")</f>
+        <f>IF(AND(G13&lt;&gt;"",UPPER(E13)="Y"),(ROUNDUP((C13-2*$M$19/12)*12/$M$18,0)+1)*((B13-2*$M$19/12)+(MAX(1,ROUNDUP(((B13-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12)+(ROUNDUP((B13-2*$M$19/12)*12/$M$18,0)+1)*((C13-2*$M$19/12)+(MAX(1,ROUNDUP(((C13-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12),"")</f>
       </c>
       <c r="L13" s="41">
+        <f>IF(AND(G13&lt;&gt;"",UPPER(E13)="Y"),(ROUNDUP((C13-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((B13-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((C13-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((B13-2*$M$19/12)-(MAX(1,ROUNDUP(((B13-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0)+(ROUNDUP((B13-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((C13-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((B13-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((C13-2*$M$19/12)-(MAX(1,ROUNDUP(((C13-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0),"")</f>
+      </c>
+      <c r="M13" s="41">
         <f>IF(OR(G13="",N(F13)&lt;=0),"",(ROUNDUP(B13/F13,0)-1)*C13+(ROUNDUP(C13/F13,0)-1)*B13)</f>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="38"/>
       <c r="B14" s="39"/>
       <c r="C14" s="39"/>
@@ -2444,18 +2476,21 @@
         <f>IF(G14="","",2*(B14+C14))</f>
       </c>
       <c r="J14" s="43">
-        <f>IF(AND(G14&lt;&gt;"",UPPER(E14)="Y"),(ROUNDUP((C14-2*$L$19/12)*12/$L$18,0)+1)&amp;" / "&amp;(ROUNDUP((B14-2*$L$19/12)*12/$L$18,0)+1),"")</f>
+        <f>IF(AND(G14&lt;&gt;"",UPPER(E14)="Y"),(ROUNDUP((C14-2*$M$19/12)*12/$M$18,0)+1)&amp;" / "&amp;(ROUNDUP((B14-2*$M$19/12)*12/$M$18,0)+1),"")</f>
       </c>
       <c r="K14" s="41">
-        <f>IF(AND(G14&lt;&gt;"",UPPER(E14)="Y"),(ROUNDUP((C14-2*$L$19/12)*12/$L$18,0)+1)*((B14-2*$L$19/12)+(MAX(1,ROUNDUP(((B14-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12)+(ROUNDUP((B14-2*$L$19/12)*12/$L$18,0)+1)*((C14-2*$L$19/12)+(MAX(1,ROUNDUP(((C14-2*$L$19/12)-$L$21/12)/($L$20-$L$21/12),0))-1)*$L$21/12),"")</f>
+        <f>IF(AND(G14&lt;&gt;"",UPPER(E14)="Y"),(ROUNDUP((C14-2*$M$19/12)*12/$M$18,0)+1)*((B14-2*$M$19/12)+(MAX(1,ROUNDUP(((B14-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12)+(ROUNDUP((B14-2*$M$19/12)*12/$M$18,0)+1)*((C14-2*$M$19/12)+(MAX(1,ROUNDUP(((C14-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*$M$21/12),"")</f>
       </c>
       <c r="L14" s="41">
+        <f>IF(AND(G14&lt;&gt;"",UPPER(E14)="Y"),(ROUNDUP((C14-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((B14-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((C14-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((B14-2*$M$19/12)-(MAX(1,ROUNDUP(((B14-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0)+(ROUNDUP((B14-2*$M$19/12)*12/$M$18,0)+1)*(MAX(1,ROUNDUP(((C14-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)+ROUNDUP((ROUNDUP((B14-2*$M$19/12)*12/$M$18,0)+1)/INT($M$20/((C14-2*$M$19/12)-(MAX(1,ROUNDUP(((C14-2*$M$19/12)-$M$21/12)/($M$20-$M$21/12),0))-1)*($M$20-$M$21/12))+1E-9),0),"")</f>
+      </c>
+      <c r="M14" s="41">
         <f>IF(OR(G14="",N(F14)&lt;=0),"",(ROUNDUP(B14/F14,0)-1)*C14+(ROUNDUP(C14/F14,0)-1)*B14)</f>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
@@ -2478,15 +2513,18 @@
       <c r="L15" s="44">
         <f>SUM(L7:L14)</f>
       </c>
+      <c r="M15" s="44">
+        <f>SUM(M7:M14)</f>
+      </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -2496,19 +2534,20 @@
         <v>0.08</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
-      <c r="L18" s="46">
+      <c r="L18" s="8"/>
+      <c r="M18" s="46">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -2518,19 +2557,20 @@
         <v>10</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
-      <c r="L19" s="47">
+      <c r="L19" s="8"/>
+      <c r="M19" s="47">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -2540,19 +2580,20 @@
         <v>4</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
-      <c r="L20" s="46">
+      <c r="L20" s="8"/>
+      <c r="M20" s="46">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -2562,19 +2603,20 @@
         <v>1.9</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
-      <c r="L21" s="46">
+      <c r="L21" s="8"/>
+      <c r="M21" s="46">
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -2584,19 +2626,20 @@
         <v>1152</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
-      <c r="L22" s="46">
+      <c r="L22" s="8"/>
+      <c r="M22" s="46">
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -2606,19 +2649,20 @@
         <v>4</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H23" s="8"/>
       <c r="I23" s="8"/>
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
-      <c r="L23" s="47">
+      <c r="L23" s="8"/>
+      <c r="M23" s="47">
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -2628,19 +2672,20 @@
         <v>145</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
-      <c r="L24" s="46">
+      <c r="L24" s="8"/>
+      <c r="M24" s="46">
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -2650,24 +2695,25 @@
         <v>150</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H25" s="8"/>
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
-      <c r="L25" s="46">
+      <c r="L25" s="8"/>
+      <c r="M25" s="46">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -2679,13 +2725,14 @@
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
-      <c r="L28" s="49">
+      <c r="L28" s="8"/>
+      <c r="M28" s="49">
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -2697,13 +2744,14 @@
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
-      <c r="L29" s="49">
+      <c r="L29" s="8"/>
+      <c r="M29" s="49">
         <v>60</v>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B31" s="13" t="s">
         <v>34</v>
@@ -2732,16 +2780,19 @@
       <c r="J31" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="K31" s="12" t="s">
+      <c r="K31" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="L31" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="L31" s="14" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M31" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="50" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B32" s="50"/>
       <c r="C32" s="50"/>
@@ -2752,16 +2803,17 @@
       <c r="H32" s="50"/>
       <c r="I32" s="50"/>
       <c r="J32" s="50"/>
-      <c r="K32" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="L32" s="52">
+      <c r="K32" s="50"/>
+      <c r="L32" s="51" t="s">
+        <v>104</v>
+      </c>
+      <c r="M32" s="52">
         <f>H15</f>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="50" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B33" s="50"/>
       <c r="C33" s="50"/>
@@ -2772,16 +2824,17 @@
       <c r="H33" s="50"/>
       <c r="I33" s="50"/>
       <c r="J33" s="50"/>
-      <c r="K33" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="L33" s="52">
+      <c r="K33" s="50"/>
+      <c r="L33" s="51" t="s">
+        <v>104</v>
+      </c>
+      <c r="M33" s="52">
         <f>ROUNDUP(H15*(1+$F$18)*4,0)/4</f>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="50" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B34" s="50"/>
       <c r="C34" s="50"/>
@@ -2792,16 +2845,17 @@
       <c r="H34" s="50"/>
       <c r="I34" s="50"/>
       <c r="J34" s="50"/>
-      <c r="K34" s="51" t="s">
-        <v>106</v>
-      </c>
-      <c r="L34" s="53">
-        <f>ROUNDUP(L33/$F$19,0)</f>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K34" s="50"/>
+      <c r="L34" s="51" t="s">
+        <v>107</v>
+      </c>
+      <c r="M34" s="53">
+        <f>ROUNDUP(M33/$F$19,0)</f>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="50" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B35" s="50"/>
       <c r="C35" s="50"/>
@@ -2812,16 +2866,17 @@
       <c r="H35" s="50"/>
       <c r="I35" s="50"/>
       <c r="J35" s="50"/>
-      <c r="K35" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="L35" s="52">
-        <f>IF(L34=0,0,L33-(L34-1)*$F$19)</f>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K35" s="50"/>
+      <c r="L35" s="51" t="s">
+        <v>104</v>
+      </c>
+      <c r="M35" s="52">
+        <f>IF(M34=0,0,M33-(M34-1)*$F$19)</f>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="50" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B36" s="50"/>
       <c r="C36" s="50"/>
@@ -2832,16 +2887,17 @@
       <c r="H36" s="50"/>
       <c r="I36" s="50"/>
       <c r="J36" s="50"/>
-      <c r="K36" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="L36" s="52">
+      <c r="K36" s="50"/>
+      <c r="L36" s="51" t="s">
+        <v>104</v>
+      </c>
+      <c r="M36" s="52">
         <f>G15*$F$20/12/27</f>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="50" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B37" s="50"/>
       <c r="C37" s="50"/>
@@ -2852,16 +2908,17 @@
       <c r="H37" s="50"/>
       <c r="I37" s="50"/>
       <c r="J37" s="50"/>
-      <c r="K37" s="51" t="s">
-        <v>110</v>
-      </c>
-      <c r="L37" s="53">
-        <f>ROUNDUP(L36*$F$21,0)</f>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K37" s="50"/>
+      <c r="L37" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="M37" s="53">
+        <f>ROUNDUP(M36*$F$21,0)</f>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="50" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B38" s="50"/>
       <c r="C38" s="50"/>
@@ -2872,16 +2929,17 @@
       <c r="H38" s="50"/>
       <c r="I38" s="50"/>
       <c r="J38" s="50"/>
-      <c r="K38" s="51" t="s">
-        <v>110</v>
-      </c>
-      <c r="L38" s="54">
+      <c r="K38" s="50"/>
+      <c r="L38" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="M38" s="54">
         <f>ROUND($F$22*$F$23/12*$F$24/2000,1)</f>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="50" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B39" s="50"/>
       <c r="C39" s="50"/>
@@ -2892,16 +2950,17 @@
       <c r="H39" s="50"/>
       <c r="I39" s="50"/>
       <c r="J39" s="50"/>
-      <c r="K39" s="51" t="s">
-        <v>113</v>
-      </c>
-      <c r="L39" s="53">
+      <c r="K39" s="50"/>
+      <c r="L39" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="M39" s="53">
         <f>K15</f>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="50" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B40" s="50"/>
       <c r="C40" s="50"/>
@@ -2912,16 +2971,17 @@
       <c r="H40" s="50"/>
       <c r="I40" s="50"/>
       <c r="J40" s="50"/>
-      <c r="K40" s="51" t="s">
-        <v>115</v>
-      </c>
-      <c r="L40" s="53">
-        <f>ROUNDUP(K15/$L$20,0)</f>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K40" s="50"/>
+      <c r="L40" s="51" t="s">
+        <v>116</v>
+      </c>
+      <c r="M40" s="53">
+        <f>L15</f>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="50" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B41" s="50"/>
       <c r="C41" s="50"/>
@@ -2932,16 +2992,17 @@
       <c r="H41" s="50"/>
       <c r="I41" s="50"/>
       <c r="J41" s="50"/>
-      <c r="K41" s="51" t="s">
-        <v>117</v>
-      </c>
-      <c r="L41" s="53">
-        <f>ROUNDUP(SUMIF(E7:E14,"Y",G7:G14)/$L$22,0)</f>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K41" s="50"/>
+      <c r="L41" s="51" t="s">
+        <v>118</v>
+      </c>
+      <c r="M41" s="53">
+        <f>ROUNDUP(SUMIF(E7:E14,"Y",G7:G14)/$M$22,0)</f>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="50" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B42" s="50"/>
       <c r="C42" s="50"/>
@@ -2952,16 +3013,17 @@
       <c r="H42" s="50"/>
       <c r="I42" s="50"/>
       <c r="J42" s="50"/>
-      <c r="K42" s="51" t="s">
-        <v>113</v>
-      </c>
-      <c r="L42" s="53">
-        <f>MAX(0,I15-L28)</f>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K42" s="50"/>
+      <c r="L42" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="M42" s="53">
+        <f>MAX(0,I15-M28)</f>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="50" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B43" s="50"/>
       <c r="C43" s="50"/>
@@ -2972,16 +3034,17 @@
       <c r="H43" s="50"/>
       <c r="I43" s="50"/>
       <c r="J43" s="50"/>
-      <c r="K43" s="51" t="s">
-        <v>117</v>
-      </c>
-      <c r="L43" s="53">
-        <f>ROUNDUP(L42/$L$23,0)</f>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K43" s="50"/>
+      <c r="L43" s="51" t="s">
+        <v>118</v>
+      </c>
+      <c r="M43" s="53">
+        <f>ROUNDUP(M42/$M$23,0)</f>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="50" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B44" s="50"/>
       <c r="C44" s="50"/>
@@ -2992,16 +3055,17 @@
       <c r="H44" s="50"/>
       <c r="I44" s="50"/>
       <c r="J44" s="50"/>
-      <c r="K44" s="51" t="s">
-        <v>115</v>
-      </c>
-      <c r="L44" s="53">
-        <f>ROUNDUP(L28/$L$24,0)</f>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K44" s="50"/>
+      <c r="L44" s="51" t="s">
+        <v>116</v>
+      </c>
+      <c r="M44" s="53">
+        <f>ROUNDUP(M28/$M$24,0)</f>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="50" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B45" s="50"/>
       <c r="C45" s="50"/>
@@ -3012,16 +3076,17 @@
       <c r="H45" s="50"/>
       <c r="I45" s="50"/>
       <c r="J45" s="50"/>
-      <c r="K45" s="51" t="s">
-        <v>113</v>
-      </c>
-      <c r="L45" s="53">
-        <f>L15</f>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K45" s="50"/>
+      <c r="L45" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="M45" s="53">
+        <f>M15</f>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="50" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B46" s="50"/>
       <c r="C46" s="50"/>
@@ -3032,16 +3097,17 @@
       <c r="H46" s="50"/>
       <c r="I46" s="50"/>
       <c r="J46" s="50"/>
-      <c r="K46" s="51" t="s">
-        <v>123</v>
-      </c>
-      <c r="L46" s="53">
-        <f>ROUNDUP(G15*$L$25/$F$25,0)</f>
-      </c>
-    </row>
-    <row r="48" ht="44" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K46" s="50"/>
+      <c r="L46" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="M46" s="53">
+        <f>ROUNDUP(G15*$M$25/$F$25,0)</f>
+      </c>
+    </row>
+    <row r="48" ht="56" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="36" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B48" s="36"/>
       <c r="C48" s="36"/>
@@ -3054,10 +3120,11 @@
       <c r="J48" s="36"/>
       <c r="K48" s="36"/>
       <c r="L48" s="36"/>
-    </row>
-    <row r="50" ht="32" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M48" s="36"/>
+    </row>
+    <row r="50" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="36" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B50" s="36"/>
       <c r="C50" s="36"/>
@@ -3070,10 +3137,11 @@
       <c r="J50" s="36"/>
       <c r="K50" s="36"/>
       <c r="L50" s="36"/>
-    </row>
-    <row r="52" ht="26" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M50" s="36"/>
+    </row>
+    <row r="52" ht="16" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B52" s="37"/>
       <c r="C52" s="37"/>
@@ -3086,45 +3154,46 @@
       <c r="J52" s="37"/>
       <c r="K52" s="37"/>
       <c r="L52" s="37"/>
+      <c r="M52" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="36">
     <mergeCell ref="A18:E18"/>
-    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="G18:L18"/>
     <mergeCell ref="A19:E19"/>
-    <mergeCell ref="G19:K19"/>
+    <mergeCell ref="G19:L19"/>
     <mergeCell ref="A20:E20"/>
-    <mergeCell ref="G20:K20"/>
+    <mergeCell ref="G20:L20"/>
     <mergeCell ref="A21:E21"/>
-    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G21:L21"/>
     <mergeCell ref="A22:E22"/>
-    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G22:L22"/>
     <mergeCell ref="A23:E23"/>
-    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G23:L23"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G24:L24"/>
     <mergeCell ref="A25:E25"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="A28:K28"/>
-    <mergeCell ref="A29:K29"/>
-    <mergeCell ref="A32:J32"/>
-    <mergeCell ref="A33:J33"/>
-    <mergeCell ref="A34:J34"/>
-    <mergeCell ref="A35:J35"/>
-    <mergeCell ref="A36:J36"/>
-    <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A38:J38"/>
-    <mergeCell ref="A39:J39"/>
-    <mergeCell ref="A40:J40"/>
-    <mergeCell ref="A41:J41"/>
-    <mergeCell ref="A42:J42"/>
-    <mergeCell ref="A43:J43"/>
-    <mergeCell ref="A44:J44"/>
-    <mergeCell ref="A45:J45"/>
-    <mergeCell ref="A46:J46"/>
-    <mergeCell ref="A48:L48"/>
-    <mergeCell ref="A50:L50"/>
-    <mergeCell ref="A52:L52"/>
+    <mergeCell ref="G25:L25"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A32:K32"/>
+    <mergeCell ref="A33:K33"/>
+    <mergeCell ref="A34:K34"/>
+    <mergeCell ref="A35:K35"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="A38:K38"/>
+    <mergeCell ref="A39:K39"/>
+    <mergeCell ref="A40:K40"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A45:K45"/>
+    <mergeCell ref="A46:K46"/>
+    <mergeCell ref="A48:M48"/>
+    <mergeCell ref="A50:M50"/>
+    <mergeCell ref="A52:M52"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Pick from the list" error="Choose one of: Y, N" sqref="E7:E14">
@@ -3162,12 +3231,12 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" ht="6" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3188,7 +3257,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -3198,7 +3267,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -3208,7 +3277,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -3218,36 +3287,36 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>29</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C11" s="20">
         <v>0</v>
@@ -3270,10 +3339,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="B12" s="19" t="s">
         <v>141</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>140</v>
       </c>
       <c r="C12" s="20">
         <v>0</v>
@@ -3296,10 +3365,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C13" s="20">
         <v>30</v>
@@ -3322,10 +3391,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C14" s="20">
         <v>0.6</v>
@@ -3348,10 +3417,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C15" s="20">
         <v>0.8</v>
@@ -3374,10 +3443,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C16" s="20">
         <v>178</v>
@@ -3400,10 +3469,10 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C17" s="20">
         <v>0.08</v>
@@ -3426,10 +3495,10 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C18" s="20">
         <v>0</v>
@@ -3548,7 +3617,7 @@
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="36" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B26" s="36"/>
       <c r="C26" s="36"/>
@@ -3560,7 +3629,7 @@
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="36" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B28" s="36"/>
       <c r="C28" s="36"/>
@@ -3572,7 +3641,7 @@
     </row>
     <row r="30" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="37" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B30" s="37"/>
       <c r="C30" s="37"/>
@@ -3618,7 +3687,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" ht="6" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -3627,103 +3696,103 @@
     </row>
     <row r="4" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="57" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B4" s="58" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="57" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B5" s="58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="57" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="57" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B7" s="58" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="57" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B8" s="58" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="57" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B9" s="58" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="59" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B12" s="60" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="59" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B13" s="60" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="59" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B14" s="60" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="59" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B15" s="60" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="36" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B17" s="36"/>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="61" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" ht="78" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="37" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B20" s="37"/>
     </row>

</xml_diff>